<commit_message>
updated for second norming study, requires debug
</commit_message>
<xml_diff>
--- a/normstim.xlsx
+++ b/normstim.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rubydowling/Documents/GitHub/norming_study_template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ADCEC23-51E2-BF41-BF2E-C33A24CD217F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{452EA078-8134-D642-BE49-A439DCBDC1DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1360" yWindow="820" windowWidth="28040" windowHeight="17060" xr2:uid="{8A491E57-1C6C-9A4D-8F9C-C69C138FA055}"/>
   </bookViews>
@@ -80,30 +80,12 @@
     <t>The baker is composed of ice cream and meringue</t>
   </si>
   <si>
-    <t>The dancer includes Spanish flamenco </t>
-  </si>
-  <si>
-    <t>The intricate competition routine includes Spanish flamenco</t>
-  </si>
-  <si>
     <t>The environmentalist runs on clean energy</t>
   </si>
   <si>
     <t>The car runs on clean energy</t>
   </si>
   <si>
-    <t>The astronomer orbits the newly discovered planet</t>
-  </si>
-  <si>
-    <t>The moon orbits the newly discovered planet</t>
-  </si>
-  <si>
-    <t>The cartographer borders the coral reef</t>
-  </si>
-  <si>
-    <t>The new island borders the coral reef</t>
-  </si>
-  <si>
     <t>The coach totals eight athletes</t>
   </si>
   <si>
@@ -116,12 +98,6 @@
     <t>The new dormitory houses only international students</t>
   </si>
   <si>
-    <t>The man encloses the backyard</t>
-  </si>
-  <si>
-    <t>The old fence encloses the backyard</t>
-  </si>
-  <si>
     <t>The queen spans the peaceful countryside</t>
   </si>
   <si>
@@ -213,6 +189,30 @@
   </si>
   <si>
     <t>The blank the painter canvas admires</t>
+  </si>
+  <si>
+    <t>The student is derived from ancient Greek texts</t>
+  </si>
+  <si>
+    <t>The tome is derived from ancient Greek texts</t>
+  </si>
+  <si>
+    <t>The artist is formed from slippery red clay</t>
+  </si>
+  <si>
+    <t>The artisan flowerpot is formed from slippery red clay</t>
+  </si>
+  <si>
+    <t>The salesman is built from the ruins of the town hall</t>
+  </si>
+  <si>
+    <t>The new skyscraper is built from the ruins of the town hall</t>
+  </si>
+  <si>
+    <t>The teacher comprises six difficult classes</t>
+  </si>
+  <si>
+    <t>The busy schedule comprises six difficult classes</t>
   </si>
 </sst>
 </file>
@@ -730,7 +730,7 @@
         <v>6</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="E8" t="s">
         <v>11</v>
@@ -747,7 +747,7 @@
         <v>8</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>15</v>
+        <v>52</v>
       </c>
       <c r="E9" t="s">
         <v>11</v>
@@ -764,7 +764,7 @@
         <v>6</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E10" t="s">
         <v>11</v>
@@ -781,7 +781,7 @@
         <v>8</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E11" t="s">
         <v>11</v>
@@ -798,7 +798,7 @@
         <v>6</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="E12" t="s">
         <v>11</v>
@@ -815,7 +815,7 @@
         <v>8</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>19</v>
+        <v>54</v>
       </c>
       <c r="E13" t="s">
         <v>11</v>
@@ -832,7 +832,7 @@
         <v>6</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="E14" t="s">
         <v>11</v>
@@ -849,7 +849,7 @@
         <v>8</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>21</v>
+        <v>56</v>
       </c>
       <c r="E15" t="s">
         <v>11</v>
@@ -866,7 +866,7 @@
         <v>6</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="E16" t="s">
         <v>11</v>
@@ -883,7 +883,7 @@
         <v>8</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="E17" t="s">
         <v>11</v>
@@ -900,7 +900,7 @@
         <v>6</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E18" t="s">
         <v>11</v>
@@ -917,7 +917,7 @@
         <v>8</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E19" t="s">
         <v>11</v>
@@ -934,7 +934,7 @@
         <v>6</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="E20" t="s">
         <v>11</v>
@@ -951,7 +951,7 @@
         <v>8</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="E21" t="s">
         <v>11</v>
@@ -968,7 +968,7 @@
         <v>6</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="E22" t="s">
         <v>11</v>
@@ -985,7 +985,7 @@
         <v>8</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="E23" t="s">
         <v>11</v>
@@ -1002,7 +1002,7 @@
         <v>6</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="E24" t="s">
         <v>11</v>
@@ -1019,7 +1019,7 @@
         <v>8</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="E25" t="s">
         <v>11</v>
@@ -1033,13 +1033,13 @@
         <v>1001</v>
       </c>
       <c r="C26" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="E26" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
@@ -1050,13 +1050,13 @@
         <v>1002</v>
       </c>
       <c r="C27" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="E27" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
@@ -1067,13 +1067,13 @@
         <v>1003</v>
       </c>
       <c r="C28" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="E28" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
@@ -1084,13 +1084,13 @@
         <v>1004</v>
       </c>
       <c r="C29" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="E29" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
@@ -1101,13 +1101,13 @@
         <v>1005</v>
       </c>
       <c r="C30" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="E30" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -1118,13 +1118,13 @@
         <v>1006</v>
       </c>
       <c r="C31" t="s">
+        <v>24</v>
+      </c>
+      <c r="D31" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D31" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="E31" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
@@ -1135,13 +1135,13 @@
         <v>1007</v>
       </c>
       <c r="C32" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="E32" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
@@ -1152,13 +1152,13 @@
         <v>1008</v>
       </c>
       <c r="C33" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E33" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
@@ -1169,13 +1169,13 @@
         <v>1009</v>
       </c>
       <c r="C34" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="E34" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
@@ -1186,13 +1186,13 @@
         <v>1010</v>
       </c>
       <c r="C35" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="E35" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
@@ -1203,13 +1203,13 @@
         <v>1011</v>
       </c>
       <c r="C36" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="E36" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
@@ -1220,13 +1220,13 @@
         <v>1012</v>
       </c>
       <c r="C37" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E37" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
@@ -1237,13 +1237,13 @@
         <v>1013</v>
       </c>
       <c r="C38" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="E38" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
@@ -1254,13 +1254,13 @@
         <v>1014</v>
       </c>
       <c r="C39" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="E39" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
@@ -1271,13 +1271,13 @@
         <v>1015</v>
       </c>
       <c r="C40" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="E40" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
@@ -1288,13 +1288,13 @@
         <v>1016</v>
       </c>
       <c r="C41" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="E41" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
@@ -1305,13 +1305,13 @@
         <v>1017</v>
       </c>
       <c r="C42" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="E42" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
@@ -1322,13 +1322,13 @@
         <v>1018</v>
       </c>
       <c r="C43" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="E43" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
@@ -1339,13 +1339,13 @@
         <v>1019</v>
       </c>
       <c r="C44" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="E44" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
@@ -1356,13 +1356,13 @@
         <v>1020</v>
       </c>
       <c r="C45" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="E45" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
@@ -1373,13 +1373,13 @@
         <v>1021</v>
       </c>
       <c r="C46" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E46" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
@@ -1390,13 +1390,13 @@
         <v>1022</v>
       </c>
       <c r="C47" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="E47" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
@@ -1407,13 +1407,13 @@
         <v>1023</v>
       </c>
       <c r="C48" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="E48" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
@@ -1424,13 +1424,13 @@
         <v>1024</v>
       </c>
       <c r="C49" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="E49" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>